<commit_message>
updated script for docker compose
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -3,13 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{2E7AF595-F8A7-41FF-83FF-C1E30967CC9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{742504F8-9393-4CD2-9E85-51E7CEEFB157}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="inValidData" sheetId="2" r:id="rId2"/>
+    <sheet name="inValidLoginData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
   <oleSize ref="A1:L16"/>

</xml_diff>